<commit_message>
Phase 2 (WIP): tests and docs in progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LC5pqG8CcTPRhQyBKryEJ8
</commit_message>
<xml_diff>
--- a/templates/SolidPro_CC_Financials_Template.xlsx
+++ b/templates/SolidPro_CC_Financials_Template.xlsx
@@ -20,14 +20,14 @@
     <comment ref="A1" authorId="0">
       <text>
         <r>
-          <t>Required: Must exist in the master</t>
+          <t>Required: Must exist in the master. Every upload REPLACES all lines for every period it contains — include every cost centre for that period.</t>
         </r>
       </text>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
         <r>
-          <t>Required: YYYY-MM</t>
+          <t>Required: YYYY-MM (or Oct-2026). One file may hold several periods, e.g. a month of actuals or a full-year budget.</t>
         </r>
       </text>
     </comment>
@@ -48,7 +48,7 @@
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>Required: Number, no currency symbols</t>
+          <t>Required: Number. Leave blank ONLY for budget-only (future) months; in a month with actuals enter 0, not blank. CC actuals per period must equal the trial balance.</t>
         </r>
       </text>
     </comment>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
   <si>
     <t>CC_Code</t>
   </si>
@@ -98,7 +98,7 @@
     <t>158400</t>
   </si>
   <si>
-    <t>SolidPro Cost Centre Portal — Budget &amp; Actuals (Phase 2) template</t>
+    <t>SolidPro Cost Centre Portal — Budget &amp; Actuals template</t>
   </si>
   <si>
     <t>Replace the example rows on the first sheet. Keep the header row unchanged. The upload is rejected as a whole if any row has an error.</t>
@@ -116,16 +116,19 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>Must exist in the master</t>
-  </si>
-  <si>
-    <t>YYYY-MM</t>
+    <t>Must exist in the master. Every upload REPLACES all lines for every period it contains — include every cost centre for that period.</t>
+  </si>
+  <si>
+    <t>YYYY-MM (or Oct-2026). One file may hold several periods, e.g. a month of actuals or a full-year budget.</t>
   </si>
   <si>
     <t>GL group as mapped from the Tally export</t>
   </si>
   <si>
     <t>Number, no currency symbols</t>
+  </si>
+  <si>
+    <t>Number. Leave blank ONLY for budget-only (future) months; in a month with actuals enter 0, not blank. CC actuals per period must equal the trial balance.</t>
   </si>
 </sst>
 </file>
@@ -672,7 +675,7 @@
         <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phase 3: default to the latest month every entity has closed; docs
- Default As-of month (My Cost Centres, export, commentary coverage) is
  the latest month all visible entities have closed, so an entity that
  has not closed yet is not shown as falsely under budget
- Admin reconciliation and register amounts use each entity's currency
  formatting (paise/cents kept)
- Tests for financials and allocations stale-batch guards, the audited
  period register and the per-entity default month (231 passing)
- README, admin guide, templates (incl. Allocations) updated for Phase 3

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LC5pqG8CcTPRhQyBKryEJ8
</commit_message>
<xml_diff>
--- a/templates/SolidPro_CC_Financials_Template.xlsx
+++ b/templates/SolidPro_CC_Financials_Template.xlsx
@@ -41,14 +41,14 @@
     <comment ref="D1" authorId="0">
       <text>
         <r>
-          <t>Required: Number, no currency symbols</t>
+          <t>Required: Number (commas, currency symbols and (brackets) for negatives are accepted). Required on every row — enter 0 if there is no budget.</t>
         </r>
       </text>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>Required: Number. Leave blank ONLY for budget-only (future) months; in a month with actuals enter 0, not blank. CC actuals per period must equal the trial balance.</t>
+          <t>Required: Number. Leave blank ONLY for budget-only (future) months; in a month with actuals enter 0, not blank. CC actuals per period and entity must equal that entity's trial balance.</t>
         </r>
       </text>
     </comment>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
   <si>
     <t>CC_Code</t>
   </si>
@@ -74,6 +74,42 @@
     <t>Actual</t>
   </si>
   <si>
+    <t>SolidPro Cost Centre Portal — Budget &amp; Actuals template</t>
+  </si>
+  <si>
+    <t>Enter your rows on the "Financials" sheet under the header row. Keep the header row unchanged. The upload is rejected as a whole if any row has an error.</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>Rule</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Must exist in the master. Every upload REPLACES all lines for every period it contains — include every cost centre for that period.</t>
+  </si>
+  <si>
+    <t>YYYY-MM (or Oct-2026). One file may hold several periods, e.g. a month of actuals or a full-year budget.</t>
+  </si>
+  <si>
+    <t>GL group as mapped from the Tally export</t>
+  </si>
+  <si>
+    <t>Number (commas, currency symbols and (brackets) for negatives are accepted). Required on every row — enter 0 if there is no budget.</t>
+  </si>
+  <si>
+    <t>Number. Leave blank ONLY for budget-only (future) months; in a month with actuals enter 0, not blank. CC actuals per period and entity must equal that entity's trial balance.</t>
+  </si>
+  <si>
+    <t>Example rows (for illustration only — do not copy blindly)</t>
+  </si>
+  <si>
     <t>IN-ENG-101</t>
   </si>
   <si>
@@ -96,46 +132,13 @@
   </si>
   <si>
     <t>158400</t>
-  </si>
-  <si>
-    <t>SolidPro Cost Centre Portal — Budget &amp; Actuals template</t>
-  </si>
-  <si>
-    <t>Replace the example rows on the first sheet. Keep the header row unchanged. The upload is rejected as a whole if any row has an error.</t>
-  </si>
-  <si>
-    <t>Column</t>
-  </si>
-  <si>
-    <t>Required</t>
-  </si>
-  <si>
-    <t>Rule</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Must exist in the master. Every upload REPLACES all lines for every period it contains — include every cost centre for that period.</t>
-  </si>
-  <si>
-    <t>YYYY-MM (or Oct-2026). One file may hold several periods, e.g. a month of actuals or a full-year budget.</t>
-  </si>
-  <si>
-    <t>GL group as mapped from the Tally export</t>
-  </si>
-  <si>
-    <t>Number, no currency symbols</t>
-  </si>
-  <si>
-    <t>Number. Leave blank ONLY for budget-only (future) months; in a month with actuals enter 0, not blank. CC actuals per period must equal the trial balance.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -155,6 +158,10 @@
     </font>
     <font>
       <b/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF16469D"/>
     </font>
   </fonts>
   <fills count="3">
@@ -182,13 +189,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -528,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="16" style="1" customWidth="1"/>
@@ -549,40 +557,6 @@
       </c>
       <c r="E1" s="3" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -594,7 +568,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -604,23 +578,23 @@
   <sheetData>
     <row r="1" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -628,10 +602,10 @@
         <v>0</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -639,10 +613,10 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -650,10 +624,10 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -661,10 +635,10 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -672,10 +646,66 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
         <v>18</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s">
         <v>23</v>
+      </c>
+      <c r="E14" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>